<commit_message>
DEC-073: draft wording packs 0.2 - F1 to F3 of the data check reworded
NOTE.CREDLONG discloses debts after more than five years and secured debts
(facts); NOTE.EMPLOYEES drops "(including directors)"; POL.FININST no longer
asserts only basic instruments. Still UNVERIFIED; nothing imported or verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015xhqMAWpHe6Lpv2aU45bcu
</commit_message>
<xml_diff>
--- a/docs/architecture/v2-data-check.xlsx
+++ b/docs/architecture/v2-data-check.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Thresholds: 23 items confirmed against reachable sources, 2 to check, 1 limitation.</t>
   </si>
   <si>
-    <t xml:space="preserve">Wording references: 29 rows; 1 finding, 6 to check, the rest consistent with the provision cited.</t>
+    <t xml:space="preserve">Wording references: 29 rows; 0 open finding, 4 reworded in draft 0.2 (DEC-073, to verify), 3 to check, the rest consistent with the provision cited.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources: legislation.gov.uk could not be reached from the build environment (DNS refused), nor could the professional bodies' pages directly. The thresholds were checked through web search results summarising ACCA, ICAEW and PwC guidance; the links are on each row. The statute links are to legislation.gov.uk for the verifier.</t>
@@ -79,60 +79,60 @@
     <t xml:space="preserve">F1</t>
   </si>
   <si>
-    <t xml:space="preserve">FINDING</t>
+    <t xml:space="preserve">DRAFTED</t>
   </si>
   <si>
     <t xml:space="preserve">NOTE.CREDLONG (FRS 102 1A pack)</t>
   </si>
   <si>
-    <t xml:space="preserve">The wording discloses creditors after more than one year, but the requirement it cites is debts payable after more than five years and secured debts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shoaib (content); engineering adds the facts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reword the body; add facts for debts after five years and for secured debts; re-run the wording review.</t>
+    <t xml:space="preserve">Draft 0.1 disclosed creditors after more than one year; the requirement cited is debts payable after more than five years and secured debts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering (done, draft 0.2, DEC-073); Shoaib verifies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reworded with two facts in draft 0.2; verify the wording and the Sch 1 paragraph.</t>
   </si>
   <si>
     <t xml:space="preserve">F2</t>
   </si>
   <si>
+    <t xml:space="preserve">NOTE.EMPLOYEES (both packs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"(including directors)" was true only where directors have contracts of service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bracket removed in draft 0.2; verify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POL.FININST (FRS 102 1A pack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The policy asserted only basic financial instruments for every client.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The position on other instruments is now a fact in draft 0.2; verify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F4</t>
+  </si>
+  <si>
     <t xml:space="preserve">CHECK</t>
   </si>
   <si>
-    <t xml:space="preserve">NOTE.EMPLOYEES (both packs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"(including directors)" is true only where directors have contracts of service.</t>
+    <t xml:space="preserve">BSS.MICRO, POL.COMPLIANCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The provision cited for the micro-entity statement and the FRS 102 paragraph for the compliance statement need confirming against the text.</t>
   </si>
   <si>
     <t xml:space="preserve">Shoaib (content)</t>
   </si>
   <si>
-    <t xml:space="preserve">Remove the bracket or make it a fact.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POL.FININST (FRS 102 1A pack)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The policy asserts only basic financial instruments for every client.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Make it conditional or a confirmed fact.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSS.MICRO, POL.COMPLIANCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The provision cited for the micro-entity statement and the FRS 102 paragraph for the compliance statement need confirming against the text.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Confirm and correct the citations before verifying.</t>
   </si>
   <si>
@@ -742,13 +742,13 @@
     <t xml:space="preserve">Employees</t>
   </si>
   <si>
-    <t xml:space="preserve">The average number of persons employed by the company (including directors) during the year was {{fact:employees.average}} ({{year:priorEnd}}: {{fact:employees.averagePrior}}).</t>
+    <t xml:space="preserve">The average number of persons employed by the company during the year was {{fact:employees.average}} ({{year:priorEnd}}: {{fact:employees.averagePrior}}).</t>
   </si>
   <si>
     <t xml:space="preserve">Companies Act 2006 s.411 (average number of employees), as applied to micro-entities</t>
   </si>
   <si>
-    <t xml:space="preserve">The average number of persons employed is right (s.411(1)). "(including directors)" is true only for directors employed under contracts of service (s.411(5)-(6)); a director without one is not counted. Suggest wording without the bracket, or a fact saying whether directors are included.</t>
+    <t xml:space="preserve">The average number of persons employed (s.411(1)). Draft 0.1 said "(including directors)", true only for directors employed under contracts of service (s.411(5)-(6)); draft 0.2 (DEC-073) drops the bracket. To verify.</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.legislation.gov.uk/ukpga/2006/46/section/411</t>
@@ -936,13 +936,14 @@
     <t xml:space="preserve">Financial instruments</t>
   </si>
   <si>
-    <t xml:space="preserve">The company has only basic financial instruments. Trade and other debtors and creditors, cash and bank balances, and loans are measured at transaction price and subsequently at amortised cost.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FRS 102 Section 11 (basic financial instruments)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">States the company has ONLY basic financial instruments: true for many small companies, not all. Make it conditional, or a fact the preparer confirms.</t>
+    <t xml:space="preserve">Basic financial instruments (trade and other debtors and creditors, cash and bank balances, and loans) are measured at transaction price and subsequently at amortised cost.
+{{fact:text.otherFinancialInstruments}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRS 102 Section 11 (basic financial instruments); Section 12 (other financial instruments)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft 0.1 asserted ONLY basic financial instruments for every client; draft 0.2 (DEC-073) states the basic-instrument policy and takes the position on other instruments from a fact (text.otherFinancialInstruments). To verify.</t>
   </si>
   <si>
     <t xml:space="preserve">POL.TAX</t>
@@ -996,14 +997,15 @@
     <t xml:space="preserve">Creditors: amounts falling due after more than one year</t>
   </si>
   <si>
-    <t xml:space="preserve">Amounts falling due after more than one year: {{line:B.CA1}} ({{year:priorEnd}}: {{line:B.CA1:prior}}).
-{{fact:text.securedDebts}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SI 2008/409 Sch 1 (indebtedness: amounts due after five years, security given)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The cited Sch 1 requirement is the aggregate of debts payable (or by instalments) after more than FIVE years, and debts on which security is given with its nature. The wording discloses creditors due after more than ONE year, which is a different figure. Engineering's data cannot split it today: it needs a five-year fact (or line) and the secured-debts fact, and a reworded body.</t>
+    <t xml:space="preserve">Creditors falling due after more than one year: {{line:B.CA1}} ({{year:priorEnd}}: {{line:B.CA1:prior}}).
+Debts payable, or repayable by instalments, after more than five years from the balance sheet date: {{fact:text.debtsAfterFiveYears}}
+Debts on which security has been given, and the nature of th</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SI 2008/409 Sch 1 (details of indebtedness: debts payable after more than five years; debts on which security is given and its nature)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Sch 1 requirement is the debts payable (or by instalments) after more than FIVE years and the debts on which security is given, with its nature. Draft 0.1 disclosed only the after-ONE-year figure; draft 0.2 (DEC-073) keeps that line for context and adds both disclosures from facts (text.debtsAfterFiveYears, text.securedDebts). To verify.</t>
   </si>
   <si>
     <t xml:space="preserve">SI 2008/409 Sch 1 (financial commitments, guarantees and contingencies)</t>
@@ -1235,26 +1237,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFEB9C"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -1366,7 +1368,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1387,7 +1389,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFC7CE"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1721,61 +1723,61 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>35</v>
@@ -1786,7 +1788,7 @@
         <v>36</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>37</v>
@@ -1795,7 +1797,7 @@
         <v>38</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>39</v>
@@ -1826,7 +1828,7 @@
         <v>46</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>47</v>
@@ -3827,7 +3829,7 @@
         <v>175</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>221</v>
@@ -3929,7 +3931,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>235</v>
       </c>
@@ -3948,8 +3950,8 @@
       <c r="F2" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>23</v>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>240</v>
@@ -4065,7 +4067,7 @@
         <v>263</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>264</v>
@@ -4123,7 +4125,7 @@
         <v>277</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>278</v>
@@ -4248,7 +4250,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>272</v>
       </c>
@@ -4267,8 +4269,8 @@
       <c r="F13" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>23</v>
+      <c r="G13" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>303</v>
@@ -4306,7 +4308,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>272</v>
       </c>
@@ -4325,8 +4327,8 @@
       <c r="F15" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>23</v>
+      <c r="G15" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>240</v>
@@ -4759,7 +4761,7 @@
         <v>366</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>367</v>

</xml_diff>